<commit_message>
feat: Excel daily construction log form converted from the Word template
- templates/Mau_NKTC.xlsx: 'Tinh hinh thi cong hang ngay' (sections 1-7),
  A4 portrait, Word margins, Times New Roman, 2 printed pages; date cell
  with 'Ngay dd thang mm nam yyyy' number format; weather check boxes
  driven by formulas; merged target blocks for each section
- Generator make_nktc_workbooks.py (replaces make_demo_f2.py) builds the
  template, the demo workbook and demo_f2.targets.json
- Demo daily sheet gains 'Su co, phat sinh' and 'Kien nghi' columns
- F2 smoke reads targets from JSON; covers a sheet name with diacritics
  and spaces; 11/11 steps pass on ExcelApi 1.1 and 1.17
- Spec section F2.3 documents target cells per section

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Qm2x45iMv7XQr8V7R8LvS
</commit_message>
<xml_diff>
--- a/test/fixtures/demo_f2.xlsx
+++ b/test/fixtures/demo_f2.xlsx
@@ -9,20 +9,24 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TDTC" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NK_TheoNgay" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mẫu NKTC" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Mẫu NKTC'!$A$1:$I$70</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="&quot;Ngày &quot;dd&quot; tháng &quot;mm&quot; năm &quot;yyyy"/>
+    <numFmt numFmtId="167" formatCode="0&quot;°C&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,9 +35,24 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Times New Roman"/>
       <b val="1"/>
+      <sz val="13"/>
     </font>
-    <font/>
+    <font>
+      <name val="Times New Roman"/>
+      <i val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -52,42 +71,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <bottom style="dotted"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -771,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G201"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -813,6 +833,16 @@
           <t>Nội dung nghiệm thu</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Sự cố, phát sinh</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Kiến nghị</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -844,6 +874,8 @@
         <v>3</v>
       </c>
       <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -875,6 +907,8 @@
         <v>3</v>
       </c>
       <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -906,6 +940,8 @@
         <v>3</v>
       </c>
       <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -922,7 +958,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -937,6 +973,8 @@
         <v>3</v>
       </c>
       <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -953,7 +991,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -968,6 +1006,8 @@
         <v>3</v>
       </c>
       <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -999,6 +1039,8 @@
         <v>3</v>
       </c>
       <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1030,6 +1072,8 @@
         <v>3</v>
       </c>
       <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -1061,6 +1105,8 @@
         <v>3</v>
       </c>
       <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1077,7 +1123,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1092,6 +1138,8 @@
         <v>3</v>
       </c>
       <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1108,7 +1156,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1123,6 +1171,8 @@
         <v>3</v>
       </c>
       <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -1154,6 +1204,8 @@
         <v>3</v>
       </c>
       <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -1185,6 +1237,8 @@
         <v>3</v>
       </c>
       <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -1216,6 +1270,8 @@
         <v>3</v>
       </c>
       <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1232,7 +1288,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1247,6 +1303,8 @@
         <v>3</v>
       </c>
       <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -1263,7 +1321,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1278,6 +1336,8 @@
         <v>3</v>
       </c>
       <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -1313,6 +1373,8 @@
           <t>Nghiệm thu công tác chuẩn bị mặt bằng, lán trại</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -1348,6 +1410,8 @@
         <v>5</v>
       </c>
       <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -1383,6 +1447,8 @@
         <v>5</v>
       </c>
       <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1403,7 +1469,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1418,6 +1484,8 @@
         <v>5</v>
       </c>
       <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -1438,7 +1506,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1453,6 +1521,8 @@
         <v>5</v>
       </c>
       <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1488,6 +1558,8 @@
         <v>5</v>
       </c>
       <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -1523,6 +1595,8 @@
         <v>5</v>
       </c>
       <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1558,6 +1632,8 @@
         <v>5</v>
       </c>
       <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1578,7 +1654,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1593,6 +1669,8 @@
         <v>5</v>
       </c>
       <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1613,7 +1691,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1628,6 +1706,8 @@
         <v>5</v>
       </c>
       <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -1664,6 +1744,8 @@
         <v>5</v>
       </c>
       <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -1700,6 +1782,8 @@
         <v>5</v>
       </c>
       <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1736,6 +1820,8 @@
         <v>5</v>
       </c>
       <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -1757,7 +1843,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1772,6 +1858,8 @@
         <v>5</v>
       </c>
       <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -1793,7 +1881,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1808,6 +1896,8 @@
         <v>5</v>
       </c>
       <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -1845,6 +1935,8 @@
         <v>5</v>
       </c>
       <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -1882,6 +1974,8 @@
         <v>5</v>
       </c>
       <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -1919,6 +2013,8 @@
         <v>5</v>
       </c>
       <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -1941,7 +2037,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1956,6 +2052,8 @@
         <v>5</v>
       </c>
       <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -1978,7 +2076,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1993,6 +2091,8 @@
         <v>5</v>
       </c>
       <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -2030,6 +2130,8 @@
         <v>5</v>
       </c>
       <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -2067,6 +2169,8 @@
         <v>5</v>
       </c>
       <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -2104,6 +2208,8 @@
         <v>5</v>
       </c>
       <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2126,7 +2232,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2141,6 +2247,8 @@
         <v>5</v>
       </c>
       <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -2163,7 +2271,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2178,6 +2286,8 @@
         <v>5</v>
       </c>
       <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -2215,6 +2325,8 @@
         <v>5</v>
       </c>
       <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -2252,6 +2364,8 @@
         <v>5</v>
       </c>
       <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -2289,6 +2403,8 @@
         <v>5</v>
       </c>
       <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -2311,7 +2427,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2326,6 +2442,8 @@
         <v>5</v>
       </c>
       <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -2348,7 +2466,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2363,6 +2481,8 @@
         <v>5</v>
       </c>
       <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -2400,6 +2520,8 @@
         <v>5</v>
       </c>
       <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -2437,6 +2559,8 @@
         <v>5</v>
       </c>
       <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -2474,6 +2598,8 @@
         <v>5</v>
       </c>
       <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -2496,7 +2622,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2511,6 +2637,8 @@
         <v>5</v>
       </c>
       <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -2533,7 +2661,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2548,6 +2676,8 @@
         <v>5</v>
       </c>
       <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -2585,6 +2715,8 @@
         <v>5</v>
       </c>
       <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -2624,6 +2756,16 @@
         <v>6</v>
       </c>
       <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Mưa lớn chiều, tạm dừng đào mương cáp 2 giờ.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Đề nghị TVGS kiểm tra lại cao độ đáy mương cáp đoạn băng đường.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -2663,6 +2805,8 @@
         <v>6</v>
       </c>
       <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -2687,7 +2831,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2702,6 +2846,8 @@
         <v>6</v>
       </c>
       <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -2725,7 +2871,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2740,6 +2886,8 @@
         <v>6</v>
       </c>
       <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -2778,6 +2926,8 @@
         <v>6</v>
       </c>
       <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -2816,6 +2966,8 @@
         <v>6</v>
       </c>
       <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -2853,6 +3005,8 @@
         <v>5</v>
       </c>
       <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -2875,7 +3029,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2890,6 +3044,8 @@
         <v>5</v>
       </c>
       <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -2912,7 +3068,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2927,6 +3083,8 @@
         <v>5</v>
       </c>
       <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -2964,6 +3122,8 @@
         <v>5</v>
       </c>
       <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -3001,6 +3161,8 @@
         <v>5</v>
       </c>
       <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -3038,6 +3200,8 @@
         <v>5</v>
       </c>
       <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -3060,7 +3224,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3079,6 +3243,8 @@
           <t>Nghiệm thu lắp đặt đường ống tưới, thử áp lực đường ống</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -3098,7 +3264,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3113,6 +3279,8 @@
         <v>4</v>
       </c>
       <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -3147,6 +3315,8 @@
         <v>4</v>
       </c>
       <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -3181,6 +3351,8 @@
         <v>4</v>
       </c>
       <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -3215,6 +3387,8 @@
         <v>4</v>
       </c>
       <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -3234,7 +3408,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3249,6 +3423,8 @@
         <v>4</v>
       </c>
       <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -3268,7 +3444,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3283,6 +3459,8 @@
         <v>4</v>
       </c>
       <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -3317,6 +3495,8 @@
         <v>4</v>
       </c>
       <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -3351,6 +3531,8 @@
         <v>4</v>
       </c>
       <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -3383,6 +3565,8 @@
         <v>4</v>
       </c>
       <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -3400,7 +3584,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3415,6 +3599,8 @@
         <v>4</v>
       </c>
       <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -3432,7 +3618,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3447,6 +3633,8 @@
         <v>4</v>
       </c>
       <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -3479,6 +3667,8 @@
         <v>4</v>
       </c>
       <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -3511,6 +3701,8 @@
         <v>4</v>
       </c>
       <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -3547,6 +3739,8 @@
           <t>Nghiệm thu lắp đặt thiết bị tưới tự động</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -3565,7 +3759,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3580,6 +3774,8 @@
         <v>4</v>
       </c>
       <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -3598,7 +3794,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3613,6 +3809,8 @@
         <v>4</v>
       </c>
       <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -3646,6 +3844,8 @@
         <v>4</v>
       </c>
       <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -3679,6 +3879,8 @@
         <v>4</v>
       </c>
       <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -3712,6 +3914,8 @@
         <v>4</v>
       </c>
       <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -3730,7 +3934,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3745,6 +3949,8 @@
         <v>4</v>
       </c>
       <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -3763,7 +3969,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3778,6 +3984,8 @@
         <v>4</v>
       </c>
       <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -3811,6 +4019,8 @@
         <v>4</v>
       </c>
       <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -3844,6 +4054,8 @@
         <v>4</v>
       </c>
       <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -3877,6 +4089,8 @@
         <v>4</v>
       </c>
       <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -3895,7 +4109,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3910,6 +4124,8 @@
         <v>4</v>
       </c>
       <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -3928,7 +4144,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3943,6 +4159,8 @@
         <v>4</v>
       </c>
       <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -3976,6 +4194,8 @@
         <v>4</v>
       </c>
       <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -4009,6 +4229,8 @@
         <v>4</v>
       </c>
       <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -4042,6 +4264,8 @@
         <v>4</v>
       </c>
       <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -4060,7 +4284,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4075,6 +4299,8 @@
         <v>4</v>
       </c>
       <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -4093,7 +4319,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4108,6 +4334,8 @@
         <v>4</v>
       </c>
       <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -4141,6 +4369,8 @@
         <v>4</v>
       </c>
       <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -4174,6 +4404,8 @@
         <v>4</v>
       </c>
       <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -4207,6 +4439,8 @@
         <v>4</v>
       </c>
       <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -4225,7 +4459,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4240,6 +4474,8 @@
         <v>4</v>
       </c>
       <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -4258,7 +4494,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4273,6 +4509,8 @@
         <v>4</v>
       </c>
       <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -4306,6 +4544,8 @@
         <v>4</v>
       </c>
       <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -4339,6 +4579,8 @@
         <v>4</v>
       </c>
       <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -4372,6 +4614,8 @@
         <v>4</v>
       </c>
       <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -4390,7 +4634,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -4405,6 +4649,8 @@
         <v>4</v>
       </c>
       <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -4423,7 +4669,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -4438,6 +4684,8 @@
         <v>4</v>
       </c>
       <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -4471,6 +4719,8 @@
         <v>4</v>
       </c>
       <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -4504,6 +4754,8 @@
         <v>4</v>
       </c>
       <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -4537,6 +4789,8 @@
         <v>4</v>
       </c>
       <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -4555,7 +4809,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4570,6 +4824,8 @@
         <v>4</v>
       </c>
       <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -4588,7 +4844,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4603,6 +4859,8 @@
         <v>4</v>
       </c>
       <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -4636,6 +4894,8 @@
         <v>4</v>
       </c>
       <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -4669,6 +4929,8 @@
         <v>4</v>
       </c>
       <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -4702,6 +4964,8 @@
         <v>4</v>
       </c>
       <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -4720,7 +4984,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4735,6 +4999,8 @@
         <v>4</v>
       </c>
       <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -4753,7 +5019,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4768,6 +5034,8 @@
         <v>4</v>
       </c>
       <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -4801,6 +5069,8 @@
         <v>4</v>
       </c>
       <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -4834,6 +5104,8 @@
         <v>4</v>
       </c>
       <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -4867,6 +5139,8 @@
         <v>4</v>
       </c>
       <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -4885,7 +5159,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -4900,6 +5174,8 @@
         <v>4</v>
       </c>
       <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -4918,7 +5194,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -4933,6 +5209,8 @@
         <v>4</v>
       </c>
       <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -4966,6 +5244,8 @@
         <v>4</v>
       </c>
       <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -4999,6 +5279,8 @@
         <v>4</v>
       </c>
       <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -5032,6 +5314,8 @@
         <v>4</v>
       </c>
       <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -5050,7 +5334,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5065,6 +5349,8 @@
         <v>4</v>
       </c>
       <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -5083,7 +5369,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -5098,6 +5384,8 @@
         <v>4</v>
       </c>
       <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -5131,6 +5419,8 @@
         <v>4</v>
       </c>
       <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -5164,6 +5454,8 @@
         <v>4</v>
       </c>
       <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -5197,6 +5489,8 @@
         <v>4</v>
       </c>
       <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -5215,7 +5509,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -5230,6 +5524,8 @@
         <v>4</v>
       </c>
       <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -5248,7 +5544,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -5263,6 +5559,8 @@
         <v>4</v>
       </c>
       <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -5296,6 +5594,8 @@
         <v>4</v>
       </c>
       <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -5329,6 +5629,8 @@
         <v>4</v>
       </c>
       <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -5362,6 +5664,8 @@
         <v>4</v>
       </c>
       <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -5380,7 +5684,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -5395,6 +5699,8 @@
         <v>4</v>
       </c>
       <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -5413,7 +5719,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -5428,6 +5734,8 @@
         <v>4</v>
       </c>
       <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -5461,6 +5769,8 @@
         <v>4</v>
       </c>
       <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -5494,6 +5804,8 @@
         <v>4</v>
       </c>
       <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -5527,6 +5839,8 @@
         <v>4</v>
       </c>
       <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -5547,7 +5861,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -5562,6 +5876,8 @@
         <v>5</v>
       </c>
       <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -5582,7 +5898,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -5597,6 +5913,8 @@
         <v>5</v>
       </c>
       <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -5632,6 +5950,8 @@
         <v>5</v>
       </c>
       <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -5667,6 +5987,8 @@
         <v>5</v>
       </c>
       <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -5702,6 +6024,8 @@
         <v>5</v>
       </c>
       <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -5722,7 +6046,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -5737,6 +6061,8 @@
         <v>5</v>
       </c>
       <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -5757,7 +6083,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -5772,6 +6098,8 @@
         <v>5</v>
       </c>
       <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -5807,6 +6135,8 @@
         <v>5</v>
       </c>
       <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -5842,6 +6172,8 @@
         <v>5</v>
       </c>
       <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -5877,6 +6209,8 @@
         <v>5</v>
       </c>
       <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -5897,7 +6231,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -5912,6 +6246,8 @@
         <v>5</v>
       </c>
       <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -5932,7 +6268,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -5947,6 +6283,8 @@
         <v>5</v>
       </c>
       <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -5982,6 +6320,8 @@
         <v>5</v>
       </c>
       <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -6017,6 +6357,8 @@
         <v>5</v>
       </c>
       <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -6052,6 +6394,8 @@
         <v>5</v>
       </c>
       <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -6072,7 +6416,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -6087,6 +6431,8 @@
         <v>5</v>
       </c>
       <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -6107,7 +6453,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -6122,6 +6468,8 @@
         <v>5</v>
       </c>
       <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -6157,6 +6505,8 @@
         <v>5</v>
       </c>
       <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -6192,6 +6542,8 @@
         <v>5</v>
       </c>
       <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -6227,6 +6579,8 @@
         <v>5</v>
       </c>
       <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -6247,7 +6601,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -6262,6 +6616,8 @@
         <v>5</v>
       </c>
       <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -6282,7 +6638,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -6297,6 +6653,8 @@
         <v>5</v>
       </c>
       <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -6332,6 +6690,8 @@
         <v>5</v>
       </c>
       <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -6367,6 +6727,8 @@
         <v>5</v>
       </c>
       <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -6402,6 +6764,8 @@
         <v>5</v>
       </c>
       <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -6422,7 +6786,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -6437,6 +6801,8 @@
         <v>5</v>
       </c>
       <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
@@ -6457,7 +6823,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -6472,6 +6838,8 @@
         <v>5</v>
       </c>
       <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -6507,6 +6875,8 @@
         <v>5</v>
       </c>
       <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -6542,6 +6912,8 @@
         <v>5</v>
       </c>
       <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -6577,6 +6949,8 @@
         <v>5</v>
       </c>
       <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -6597,7 +6971,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -6612,6 +6986,8 @@
         <v>5</v>
       </c>
       <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
@@ -6632,7 +7008,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -6647,6 +7023,8 @@
         <v>5</v>
       </c>
       <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -6682,6 +7060,8 @@
         <v>5</v>
       </c>
       <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -6717,6 +7097,8 @@
         <v>5</v>
       </c>
       <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -6752,6 +7134,8 @@
         <v>5</v>
       </c>
       <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -6772,7 +7156,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -6787,6 +7171,8 @@
         <v>5</v>
       </c>
       <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
@@ -6807,7 +7193,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -6822,6 +7208,8 @@
         <v>5</v>
       </c>
       <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -6857,6 +7245,8 @@
         <v>5</v>
       </c>
       <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -6892,6 +7282,8 @@
         <v>5</v>
       </c>
       <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -6927,6 +7319,8 @@
         <v>5</v>
       </c>
       <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -6947,7 +7341,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -6962,6 +7356,8 @@
         <v>5</v>
       </c>
       <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
@@ -6984,7 +7380,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -6999,6 +7395,8 @@
         <v>5</v>
       </c>
       <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
@@ -7036,6 +7434,8 @@
         <v>5</v>
       </c>
       <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
@@ -7073,6 +7473,8 @@
         <v>5</v>
       </c>
       <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -7110,6 +7512,8 @@
         <v>5</v>
       </c>
       <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
@@ -7132,7 +7536,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -7147,6 +7551,8 @@
         <v>5</v>
       </c>
       <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
@@ -7169,7 +7575,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -7184,6 +7590,8 @@
         <v>5</v>
       </c>
       <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
@@ -7221,6 +7629,8 @@
         <v>5</v>
       </c>
       <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -7258,6 +7668,8 @@
         <v>5</v>
       </c>
       <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -7295,6 +7707,8 @@
         <v>5</v>
       </c>
       <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -7317,7 +7731,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -7332,6 +7746,8 @@
         <v>5</v>
       </c>
       <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -7354,7 +7770,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -7369,6 +7785,8 @@
         <v>5</v>
       </c>
       <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
@@ -7406,6 +7824,8 @@
         <v>5</v>
       </c>
       <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
@@ -7443,6 +7863,8 @@
         <v>5</v>
       </c>
       <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr"/>
+      <c r="I193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
@@ -7480,6 +7902,8 @@
         <v>5</v>
       </c>
       <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr"/>
+      <c r="I194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -7502,7 +7926,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -7517,6 +7941,8 @@
         <v>5</v>
       </c>
       <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr"/>
+      <c r="I195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
@@ -7539,7 +7965,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -7554,6 +7980,8 @@
         <v>5</v>
       </c>
       <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr"/>
+      <c r="I196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
@@ -7591,6 +8019,8 @@
         <v>5</v>
       </c>
       <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr"/>
+      <c r="I197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
@@ -7628,6 +8058,8 @@
         <v>5</v>
       </c>
       <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr"/>
+      <c r="I198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
@@ -7665,6 +8097,8 @@
         <v>5</v>
       </c>
       <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
+      <c r="I199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
@@ -7687,7 +8121,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Mưa rào chiều</t>
+          <t>Nắng, chiều mưa rào</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -7706,6 +8140,8 @@
           <t>Nghiệm thu trồng cây xanh, bó bồn gốc cây</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr"/>
+      <c r="I200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
@@ -7722,7 +8158,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Nắng</t>
+          <t>Bình thường</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -7737,6 +8173,8 @@
         <v>3</v>
       </c>
       <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr"/>
+      <c r="I201" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7747,248 +8185,754 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="9.6" customWidth="1" min="1" max="1"/>
+    <col width="9.6" customWidth="1" min="2" max="2"/>
+    <col width="9.6" customWidth="1" min="3" max="3"/>
+    <col width="9.6" customWidth="1" min="4" max="4"/>
+    <col width="9.6" customWidth="1" min="5" max="5"/>
+    <col width="9.6" customWidth="1" min="6" max="6"/>
+    <col width="9.6" customWidth="1" min="7" max="7"/>
+    <col width="9.6" customWidth="1" min="8" max="8"/>
+    <col width="9.6" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>NHẬT KÝ THI CÔNG</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Công trình: Cảnh quan – Hạ tầng (biểu mẫu MẪU để chạy thử)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>TÌNH HÌNH THI CÔNG HÀNG NGÀY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="E2" s="4" t="n"/>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Ngày:</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Thời tiết:</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="5" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+          <t>1. Thời tiết</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="B5" s="6">
+        <f>IF(AND($C$6&lt;&gt;"",NOT(ISNUMBER(SEARCH("mưa",$C$6))),NOT(ISNUMBER(SEARCH("nắng",$C$6)))),"☒","☐")&amp;" Bình thường"</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>IF(ISNUMBER(SEARCH("mưa",$C$6)),"☒","☐")&amp;" Mưa"</f>
+        <v/>
+      </c>
+      <c r="H5" s="6">
+        <f>IF(ISNUMBER(SEARCH("nắng",$C$6)),"☒","☐")&amp;" Nắng"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Ghi chú thời tiết:</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Nhiệt độ:</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Sáng</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Trưa</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Chiều</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Tối</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="n"/>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2. Tình hình nhân lực, thiết bị thi công:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2.1. Nhân lực:</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Ban chỉ huy - CBKT:</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Số công nhân:</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Số thiết bị:</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>1. NỘI DUNG CÔNG VIỆC THỰC HIỆN</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>2. NỘI DUNG NGHIỆM THU</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="10">
-        <f>"Xác nhận nhật ký ngày "&amp;TEXT(B4,"dd/mm/yyyy")</f>
-        <v/>
-      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Số lượng công nhân:</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>người</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>2.2. Thiết bị:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Số lượng thiết bị:</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>3. Tình hình thi công:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>3.1. Nội dung, khối lượng công việc và tiến độ thực hiện:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+      <c r="H35" s="8" t="n"/>
+      <c r="I35" s="8" t="n"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="n"/>
+      <c r="H38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>3.2. Nghiệm thu công việc xây dựng hàng ngày:</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="12" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="8" t="n"/>
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="n"/>
+      <c r="H45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="n"/>
+      <c r="H46" s="8" t="n"/>
+      <c r="I46" s="8" t="n"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="8" t="n"/>
+      <c r="B47" s="8" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="8" t="n"/>
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="n"/>
+      <c r="H47" s="8" t="n"/>
+      <c r="I47" s="8" t="n"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>4. Mô tả chi tiết các sự cố, hư hỏng và các vấn đề phát sinh khác trong quá trình thi công xây dựng công trình:</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="12" t="n"/>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="8" t="n"/>
+      <c r="H51" s="8" t="n"/>
+      <c r="I51" s="8" t="n"/>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="A52" s="8" t="n"/>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
+    </row>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="8" t="n"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="n"/>
+      <c r="G53" s="8" t="n"/>
+      <c r="H53" s="8" t="n"/>
+      <c r="I53" s="8" t="n"/>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>5. Các kiến nghị và những ý kiến chỉ đạo giải quyết các vấn đề phát sinh của các bên có liên quan (Chủ đầu tư, Người giám sát thi công, Người giám sát tác giả)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="12" t="n"/>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="8" t="n"/>
+      <c r="H56" s="8" t="n"/>
+      <c r="I56" s="8" t="n"/>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="8" t="n"/>
+      <c r="E57" s="8" t="n"/>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="8" t="n"/>
+      <c r="H57" s="8" t="n"/>
+      <c r="I57" s="8" t="n"/>
+    </row>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="8" t="n"/>
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="E58" s="8" t="n"/>
+      <c r="F58" s="8" t="n"/>
+      <c r="G58" s="8" t="n"/>
+      <c r="H58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
+    </row>
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="8" t="n"/>
+      <c r="C59" s="8" t="n"/>
+      <c r="D59" s="8" t="n"/>
+      <c r="E59" s="8" t="n"/>
+      <c r="F59" s="8" t="n"/>
+      <c r="G59" s="8" t="n"/>
+      <c r="H59" s="8" t="n"/>
+      <c r="I59" s="8" t="n"/>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>6. Nhận xét của kỹ sư giám sát thi công xây dựng về tình hình và chất lượng công việc xây dựng (ghi rõ họ và tên, chức vụ và chữ ký)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="20.475" customHeight="1">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="8" t="n"/>
+      <c r="C62" s="8" t="n"/>
+      <c r="D62" s="8" t="n"/>
+      <c r="E62" s="8" t="n"/>
+      <c r="F62" s="8" t="n"/>
+      <c r="G62" s="8" t="n"/>
+      <c r="H62" s="8" t="n"/>
+      <c r="I62" s="8" t="n"/>
+    </row>
+    <row r="63" ht="20.475" customHeight="1">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="8" t="n"/>
+      <c r="C63" s="8" t="n"/>
+      <c r="D63" s="8" t="n"/>
+      <c r="E63" s="8" t="n"/>
+      <c r="F63" s="8" t="n"/>
+      <c r="G63" s="8" t="n"/>
+      <c r="H63" s="8" t="n"/>
+      <c r="I63" s="8" t="n"/>
+    </row>
+    <row r="64" ht="20.475" customHeight="1">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="n"/>
+      <c r="D64" s="8" t="n"/>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="8" t="n"/>
+      <c r="G64" s="8" t="n"/>
+      <c r="H64" s="8" t="n"/>
+      <c r="I64" s="8" t="n"/>
+    </row>
+    <row r="65" ht="20.475" customHeight="1">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="8" t="n"/>
+      <c r="C65" s="8" t="n"/>
+      <c r="D65" s="8" t="n"/>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="8" t="n"/>
+      <c r="G65" s="8" t="n"/>
+      <c r="H65" s="8" t="n"/>
+      <c r="I65" s="8" t="n"/>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>7. Chỉ huy trưởng công trường tiếp thu các kiến nghị và nhận xét (họ tên, chữ ký)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20.475" customHeight="1">
+      <c r="A67" s="8" t="n"/>
+      <c r="B67" s="8" t="n"/>
+      <c r="C67" s="8" t="n"/>
+      <c r="D67" s="8" t="n"/>
+      <c r="E67" s="8" t="n"/>
+      <c r="F67" s="8" t="n"/>
+      <c r="G67" s="8" t="n"/>
+      <c r="H67" s="8" t="n"/>
+      <c r="I67" s="8" t="n"/>
+    </row>
+    <row r="68" ht="20.475" customHeight="1">
+      <c r="A68" s="8" t="n"/>
+      <c r="B68" s="8" t="n"/>
+      <c r="C68" s="8" t="n"/>
+      <c r="D68" s="8" t="n"/>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+    </row>
+    <row r="69" ht="20.475" customHeight="1">
+      <c r="A69" s="8" t="n"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="8" t="n"/>
+      <c r="D69" s="8" t="n"/>
+      <c r="E69" s="8" t="n"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="n"/>
+    </row>
+    <row r="70" ht="20.475" customHeight="1">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="n"/>
+      <c r="D70" s="8" t="n"/>
+      <c r="E70" s="8" t="n"/>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="8" t="n"/>
+      <c r="H70" s="8" t="n"/>
+      <c r="I70" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A21:F24"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F18"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="B4:C4"/>
+  <mergeCells count="27">
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A66:I66"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="A48:I49"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="A40:I47"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A60:I61"/>
+    <mergeCell ref="A21:I38"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A54:I55"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="A56:I59"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A50:I53"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I18"/>
+    <mergeCell ref="C11:I11"/>
+    <mergeCell ref="A13:I14"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.984251968503937" right="0.7874015748031495" top="0.7874015748031495" bottom="0.7874015748031495" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="47" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>